<commit_message>
Archive COS reporting and other progress data
</commit_message>
<xml_diff>
--- a/COS Reports/cos_codebook.xlsx
+++ b/COS Reports/cos_codebook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lroesele.IVV5NET\sciebo - Röseler, Lukas (lroesele@uni-muenster.de)@uni-muenster.sciebo.de\LeaRn\FReD-data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lukaswallrich/Documents/Coding/fred_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{574F0867-2CD0-4072-805A-5C0FFA6F033E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08F65E4C-2C16-474B-A069-9773B565B229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2851DFFD-9FDA-4772-BEAF-57C4965BB55C}"/>
+    <workbookView xWindow="-36280" yWindow="-1300" windowWidth="29040" windowHeight="15720" xr2:uid="{2851DFFD-9FDA-4772-BEAF-57C4965BB55C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="83">
   <si>
     <t>ref_o</t>
   </si>
@@ -224,9 +224,6 @@
     <t>replication effect size converted to r using this function: https://forrt.org/FReD/reference/convert_effect_sizes.html</t>
   </si>
   <si>
-    <t>Link to replication results - only when DOI missing or for aggregate report</t>
-  </si>
-  <si>
     <t>How is p-val reported? "=" (e) / "&lt;" (l) / "&gt;" (g) or combined (le, ge)? for example "p &lt;= .05" is coded as "le"</t>
   </si>
   <si>
@@ -254,22 +251,7 @@
     <t>Filename of the report used to code variables from the replication study</t>
   </si>
   <si>
-    <t>replication_success</t>
-  </si>
-  <si>
     <t>Binary replication success indicator. TRUE if significant and in the same direction as the original, FALSE if not significant or in the opposite direction, NA if effects are not directionally or original was not significant</t>
-  </si>
-  <si>
-    <t>Corresponding entry in the FORRT Replication Database (FReD), can be used to pick only data from the fully validated version (this version) over the crowdsourced FReD data.</t>
-  </si>
-  <si>
-    <t>outcome</t>
-  </si>
-  <si>
-    <t>outcome_quote</t>
-  </si>
-  <si>
-    <t>out_quote_source</t>
   </si>
   <si>
     <t>Outcome statement by replication authors</t>
@@ -280,6 +262,30 @@
   </si>
   <si>
     <t>Source of the quote</t>
+  </si>
+  <si>
+    <t>reported_success</t>
+  </si>
+  <si>
+    <t>reported_success_quote</t>
+  </si>
+  <si>
+    <t>reported_success_quote_source</t>
+  </si>
+  <si>
+    <t>statistical_success</t>
+  </si>
+  <si>
+    <t>Link to replication results - only when DOI missing or where DOI refers to aggregate report</t>
+  </si>
+  <si>
+    <t>Corresponding entry in the FORRT Replication Database (FReD), can be used to filter the crowdsourced FReD data for additional studies.</t>
+  </si>
+  <si>
+    <t>fred_id_old</t>
+  </si>
+  <si>
+    <t>Less consistent version of fred_id - should only be used to combine data with earlier versions of this dataset</t>
   </si>
 </sst>
 </file>
@@ -299,11 +305,13 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -453,7 +461,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -469,7 +477,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -785,14 +793,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1DB5285-B365-4E31-B843-1F907BB019DF}">
-  <dimension ref="A1:B79"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B80"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="128.28515625" customWidth="1"/>
+    <col min="1" max="1" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="128.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>38</v>
       </c>
@@ -800,481 +808,489 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="4" t="s">
+    </row>
+    <row r="3" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>41</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="28" x14ac:dyDescent="0.2">
+      <c r="A40" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="28" x14ac:dyDescent="0.2">
+      <c r="A41" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="28" x14ac:dyDescent="0.2">
+      <c r="A42" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="28" x14ac:dyDescent="0.2">
+      <c r="A43" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B43" s="4" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="B31" s="14" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="B32" s="14" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A39" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A40" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="1"/>
-      <c r="B43" s="2"/>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" s="1"/>
       <c r="B44" s="2"/>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" s="1"/>
       <c r="B45" s="2"/>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" s="1"/>
       <c r="B46" s="2"/>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" s="1"/>
       <c r="B47" s="2"/>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" s="1"/>
       <c r="B48" s="2"/>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" s="1"/>
       <c r="B49" s="2"/>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" s="1"/>
       <c r="B50" s="2"/>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" s="1"/>
       <c r="B51" s="2"/>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" s="1"/>
       <c r="B52" s="2"/>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53" s="1"/>
       <c r="B53" s="2"/>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" s="1"/>
       <c r="B54" s="2"/>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55" s="1"/>
       <c r="B55" s="2"/>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56" s="1"/>
       <c r="B56" s="2"/>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57" s="1"/>
       <c r="B57" s="2"/>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A58" s="1"/>
       <c r="B58" s="2"/>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A59" s="1"/>
       <c r="B59" s="2"/>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A60" s="1"/>
       <c r="B60" s="2"/>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A61" s="1"/>
       <c r="B61" s="2"/>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62" s="1"/>
       <c r="B62" s="2"/>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63" s="1"/>
       <c r="B63" s="2"/>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A64" s="1"/>
       <c r="B64" s="2"/>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65" s="1"/>
       <c r="B65" s="2"/>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A66" s="1"/>
       <c r="B66" s="2"/>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A67" s="1"/>
       <c r="B67" s="2"/>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A68" s="1"/>
       <c r="B68" s="2"/>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A69" s="1"/>
       <c r="B69" s="2"/>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70" s="1"/>
       <c r="B70" s="2"/>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A71" s="1"/>
       <c r="B71" s="2"/>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A72" s="1"/>
       <c r="B72" s="2"/>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A73" s="1"/>
       <c r="B73" s="2"/>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A74" s="1"/>
       <c r="B74" s="2"/>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A75" s="1"/>
       <c r="B75" s="2"/>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A76" s="1"/>
       <c r="B76" s="2"/>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A77" s="1"/>
       <c r="B77" s="2"/>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A78" s="1"/>
       <c r="B78" s="2"/>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A79" s="1"/>
       <c r="B79" s="2"/>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A80" s="1"/>
+      <c r="B80" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>